<commit_message>
HI and summary file updates for paper writing
</commit_message>
<xml_diff>
--- a/data/constituents/raw_lab_data/phosphorus/ppdata.xlsx
+++ b/data/constituents/raw_lab_data/phosphorus/ppdata.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nicol\Documents\hysteresis\data\constituents\raw_lab_data\phosphorus\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huck4481\Documents\GitHub\hysteresis\data\constituents\raw_lab_data\phosphorus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92541F51-8ACB-44A3-93E0-576E11AF7158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3A75B3-AA94-4C1C-9631-E6D44F91528A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="7" activeTab="7" xr2:uid="{CBEDBD6E-F4C7-4255-AFE3-946B66D5A836}"/>
+    <workbookView xWindow="-25320" yWindow="360" windowWidth="25440" windowHeight="15270" activeTab="4" xr2:uid="{CBEDBD6E-F4C7-4255-AFE3-946B66D5A836}"/>
   </bookViews>
   <sheets>
     <sheet name="samples (wrong)" sheetId="1" r:id="rId1"/>
@@ -11706,7 +11706,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="16"/>
                 <c:pt idx="0">
-                  <c:v>-1.6651719999999978E-3</c:v>
+                  <c:v>-1.6651719999999999E-3</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>9.3759881818181838E-3</c:v>
@@ -37056,11 +37056,11 @@
         <v>0.6791666666666667</v>
       </c>
       <c r="C24">
-        <v>-1.6651719999999978E-3</v>
+        <v>-1.6651719999999999E-3</v>
       </c>
       <c r="D24">
         <f t="shared" si="0"/>
-        <v>5.1576641217063925E-5</v>
+        <v>5.1576641217063993E-5</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -41026,7 +41026,7 @@
         <v>0.72120350933333333</v>
       </c>
       <c r="Q4">
-        <f t="shared" ref="Q4:Q17" si="1">ABS(P4*0.030973762)</f>
+        <f t="shared" ref="Q4:Q16" si="1">ABS(P4*0.030973762)</f>
         <v>2.2338385851655443E-2</v>
       </c>
       <c r="S4" t="s">

</xml_diff>